<commit_message>
Apply human reviews and curator dataset deduplication
</commit_message>
<xml_diff>
--- a/sources/MetaVir/Plot/exposures_meta_analysis_aggressive_prostate_cancer_combined.xlsx
+++ b/sources/MetaVir/Plot/exposures_meta_analysis_aggressive_prostate_cancer_combined.xlsx
@@ -23,16 +23,13 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -52,7 +49,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -60,22 +57,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -464,57 +452,57 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Exposure</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>number studies</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Pooled RR</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>lower CI RR</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>upper CI RR</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>lower PI RR</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>upper PI RR</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>I^2 (%)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>eggers p-value</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>total N</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>total Cases</t>
         </is>
@@ -526,28 +514,28 @@
           <t>magnesium</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="3" t="n">
         <v>0.26</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="3" t="n">
         <v>0.09</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="3" t="n">
         <v>0.85</v>
       </c>
-      <c r="F2" s="4" t="inlineStr"/>
-      <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="6" t="inlineStr"/>
-      <c r="J2" s="3" t="n">
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="5" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
         <v>261</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="K2" s="2" t="n">
         <v>98</v>
       </c>
     </row>
@@ -557,28 +545,28 @@
           <t>vitamin_k2</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="3" t="n">
         <v>0.37</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="3" t="n">
         <v>0.16</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="3" t="n">
         <v>0.88</v>
       </c>
-      <c r="F3" s="4" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="6" t="inlineStr"/>
-      <c r="J3" s="3" t="n">
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="5" t="inlineStr"/>
+      <c r="J3" s="2" t="n">
         <v>11319</v>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="K3" s="2" t="n">
         <v>113</v>
       </c>
     </row>
@@ -588,28 +576,28 @@
           <t>insoluble_dietary_fiber_intake</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="3" t="n">
         <v>0.46</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="3" t="n">
         <v>0.22</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="3" t="n">
         <v>0.93</v>
       </c>
-      <c r="F4" s="4" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="6" t="inlineStr"/>
-      <c r="J4" s="3" t="n">
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
         <v>43435</v>
       </c>
-      <c r="K4" s="3" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -617,28 +605,28 @@
           <t>green_tea</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="3" t="n">
         <v>0.52</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>0.28</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="3" t="n">
         <v>0.96</v>
       </c>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="6" t="inlineStr"/>
-      <c r="J5" s="3" t="n">
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="5" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
         <v>49920</v>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="K5" s="2" t="n">
         <v>114</v>
       </c>
     </row>
@@ -648,28 +636,28 @@
           <t>inositol</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="3" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="3" t="n">
         <v>0.39</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="3" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="6" t="inlineStr"/>
-      <c r="J6" s="3" t="n">
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="2" t="n">
         <v>400</v>
       </c>
-      <c r="K6" s="3" t="n">
+      <c r="K6" s="2" t="n">
         <v>100</v>
       </c>
     </row>
@@ -679,28 +667,28 @@
           <t>beta_carotene</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="3" t="n">
         <v>0.6</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="3" t="n">
         <v>0.3</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="3" t="n">
         <v>1.6</v>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="3" t="n">
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="5" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
         <v>1037</v>
       </c>
-      <c r="K7" s="3" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -708,34 +696,34 @@
           <t>vitamin_e</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="3" t="n">
         <v>0.64</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="3" t="n">
         <v>1.04</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" s="3" t="n">
         <v>0.08</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="3" t="n">
         <v>5.21</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="4" t="n">
         <v>76.5</v>
       </c>
-      <c r="I8" s="6" t="n">
-        <v>0.2832792558734609</v>
-      </c>
-      <c r="J8" s="3" t="n">
+      <c r="I8" s="5" t="n">
+        <v>0.283279255873461</v>
+      </c>
+      <c r="J8" s="2" t="n">
         <v>114280</v>
       </c>
-      <c r="K8" s="3" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -743,34 +731,34 @@
           <t>selenium</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="3" t="n">
         <v>0.65</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="3" t="n">
         <v>0.37</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="3" t="n">
         <v>1.12</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F9" s="3" t="n">
         <v>0.09</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="G9" s="3" t="n">
         <v>4.9</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="4" t="n">
         <v>89.40000000000001</v>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="I9" s="5" t="n">
         <v>0.8385914121835617</v>
       </c>
-      <c r="J9" s="3" t="n">
+      <c r="J9" s="2" t="n">
         <v>123475</v>
       </c>
-      <c r="K9" s="3" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -778,34 +766,34 @@
           <t>lycopene</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="3" t="n">
         <v>0.67</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="3" t="n">
         <v>0.54</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="3" t="n">
         <v>0.82</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="F10" s="3" t="n">
         <v>0.16</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="3" t="n">
         <v>2.72</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="4" t="n">
         <v>3.2</v>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="I10" s="5" t="n">
         <v>0.01466213900991506</v>
       </c>
-      <c r="J10" s="3" t="n">
+      <c r="J10" s="2" t="n">
         <v>216679</v>
       </c>
-      <c r="K10" s="3" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -813,34 +801,34 @@
           <t>tomato</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="3" t="n">
         <v>0.54</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="3" t="n">
         <v>0.14</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="3" t="n">
         <v>3.54</v>
       </c>
-      <c r="H11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="6" t="n">
+      <c r="H11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5" t="n">
         <v>0.1511955352792509</v>
       </c>
-      <c r="J11" s="3" t="n">
+      <c r="J11" s="2" t="n">
         <v>124620</v>
       </c>
-      <c r="K11" s="3" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -848,28 +836,28 @@
           <t>legumes</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="3" t="n">
         <v>0.74</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="3" t="n">
         <v>0.61</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="3" t="n">
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="2" t="n">
         <v>82483</v>
       </c>
-      <c r="K12" s="3" t="n">
+      <c r="K12" s="2" t="n">
         <v>1278</v>
       </c>
     </row>
@@ -879,28 +867,28 @@
           <t>tea</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="3" t="n">
         <v>0.74</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="3" t="n">
         <v>0.44</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="3" t="n">
         <v>1.22</v>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="5" t="n">
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="4" t="n">
         <v>60.6</v>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
-      <c r="J13" s="3" t="n">
+      <c r="I13" s="5" t="inlineStr"/>
+      <c r="J13" s="2" t="n">
         <v>192116</v>
       </c>
-      <c r="K13" s="3" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -908,34 +896,34 @@
           <t>vitamin_d</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="3" t="n">
         <v>0.74</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="3" t="n">
         <v>0.51</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="3" t="n">
         <v>1.08</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="F14" s="3" t="n">
         <v>0.21</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" s="3" t="n">
         <v>2.56</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="4" t="n">
         <v>81.90000000000001</v>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="I14" s="5" t="n">
         <v>0.2069198638695529</v>
       </c>
-      <c r="J14" s="3" t="n">
+      <c r="J14" s="2" t="n">
         <v>45247</v>
       </c>
-      <c r="K14" s="3" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -943,28 +931,28 @@
           <t>folic_acid</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="3" t="n">
         <v>0.78</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="3" t="n">
         <v>0.53</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="3" t="n">
         <v>1.15</v>
       </c>
-      <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="6" t="inlineStr"/>
-      <c r="J15" s="3" t="n">
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5" t="inlineStr"/>
+      <c r="J15" s="2" t="n">
         <v>65836</v>
       </c>
-      <c r="K15" s="3" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -972,28 +960,28 @@
           <t>eicosapentaenoic_acid</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="3" t="n">
         <v>0.82</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="3" t="n">
         <v>0.64</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="3" t="n">
         <v>1.04</v>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="6" t="inlineStr"/>
-      <c r="J16" s="3" t="n">
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="2" t="n">
         <v>288268</v>
       </c>
-      <c r="K16" s="3" t="n">
+      <c r="K16" s="2" t="n">
         <v>725</v>
       </c>
     </row>
@@ -1003,28 +991,28 @@
           <t>zinc</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="3" t="n">
         <v>0.84</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="3" t="n">
         <v>0.17</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="3" t="n">
         <v>4.29</v>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="5" t="n">
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="4" t="n">
         <v>87.8</v>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="3" t="n">
+      <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="2" t="n">
         <v>82482</v>
       </c>
-      <c r="K17" s="3" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1032,28 +1020,28 @@
           <t>dash_diet</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="3" t="n">
         <v>0.86</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="3" t="n">
         <v>0.77</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="3" t="n">
         <v>0.98</v>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
-      <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="6" t="inlineStr"/>
-      <c r="J18" s="3" t="n">
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="2" t="n">
         <v>79930</v>
       </c>
-      <c r="K18" s="3" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1061,28 +1049,28 @@
           <t>total_dietary_fiber_intake</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="3" t="n">
         <v>0.86</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="3" t="n">
         <v>0.63</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="3" t="n">
         <v>1.17</v>
       </c>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="5" t="n">
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="4" t="n">
         <v>51.2</v>
       </c>
-      <c r="I19" s="6" t="inlineStr"/>
-      <c r="J19" s="3" t="n">
+      <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="2" t="n">
         <v>885584</v>
       </c>
-      <c r="K19" s="3" t="n">
+      <c r="K19" s="2" t="n">
         <v>5076</v>
       </c>
     </row>
@@ -1092,28 +1080,28 @@
           <t>mediterranean_diet</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="3" t="n">
         <v>1.02</v>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="D20" s="3" t="n">
         <v>0.92</v>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" s="3" t="n">
         <v>1.13</v>
       </c>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="5" t="n">
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
-      <c r="J20" s="3" t="n">
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
         <v>106146</v>
       </c>
-      <c r="K20" s="3" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1121,34 +1109,34 @@
           <t>betaine</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="3" t="n">
         <v>1.03</v>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" s="3" t="n">
         <v>0.6</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="3" t="n">
         <v>1.74</v>
       </c>
-      <c r="F21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="4" t="n">
+      <c r="F21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3" t="n">
         <v>503.47</v>
       </c>
-      <c r="H21" s="5" t="n">
+      <c r="H21" s="4" t="n">
         <v>76.2</v>
       </c>
-      <c r="I21" s="6" t="n">
-        <v>0.9557907411725424</v>
-      </c>
-      <c r="J21" s="3" t="n">
+      <c r="I21" s="5" t="n">
+        <v>0.9557907411725423</v>
+      </c>
+      <c r="J21" s="2" t="n">
         <v>55116</v>
       </c>
-      <c r="K21" s="3" t="n">
+      <c r="K21" s="2" t="n">
         <v>963</v>
       </c>
     </row>
@@ -1158,28 +1146,28 @@
           <t>gondoic_acid</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="C22" s="3" t="n">
         <v>1.05</v>
       </c>
-      <c r="D22" s="4" t="n">
+      <c r="D22" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="E22" s="3" t="n">
         <v>1.11</v>
       </c>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr"/>
-      <c r="H22" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="6" t="inlineStr"/>
-      <c r="J22" s="3" t="n">
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="5" t="inlineStr"/>
+      <c r="J22" s="2" t="n">
         <v>142239</v>
       </c>
-      <c r="K22" s="3" t="n">
+      <c r="K22" s="2" t="n">
         <v>936</v>
       </c>
     </row>
@@ -1189,28 +1177,28 @@
           <t>butyric_acid</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="3" t="n">
         <v>1.08</v>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="D23" s="3" t="n">
         <v>1.01</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="3" t="n">
         <v>1.15</v>
       </c>
-      <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="6" t="inlineStr"/>
-      <c r="J23" s="3" t="n">
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="5" t="inlineStr"/>
+      <c r="J23" s="2" t="n">
         <v>142239</v>
       </c>
-      <c r="K23" s="3" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1218,28 +1206,28 @@
           <t>western_pattern_diet</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="C24" s="3" t="n">
         <v>1.23</v>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="D24" s="3" t="n">
         <v>0.82</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" s="3" t="n">
         <v>1.84</v>
       </c>
-      <c r="F24" s="4" t="inlineStr"/>
-      <c r="G24" s="4" t="inlineStr"/>
-      <c r="H24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="6" t="inlineStr"/>
-      <c r="J24" s="3" t="n">
+      <c r="F24" s="3" t="inlineStr"/>
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="5" t="inlineStr"/>
+      <c r="J24" s="2" t="n">
         <v>43469</v>
       </c>
-      <c r="K24" s="3" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1247,28 +1235,28 @@
           <t>plant_protein_intake</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C25" s="3" t="n">
         <v>1.24</v>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="D25" s="3" t="n">
         <v>1.04</v>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="E25" s="3" t="n">
         <v>1.47</v>
       </c>
-      <c r="F25" s="4" t="inlineStr"/>
-      <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="6" t="inlineStr"/>
-      <c r="J25" s="3" t="n">
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="5" t="inlineStr"/>
+      <c r="J25" s="2" t="n">
         <v>150671</v>
       </c>
-      <c r="K25" s="3" t="n">
+      <c r="K25" s="2" t="n">
         <v>2170</v>
       </c>
     </row>
@@ -1278,28 +1266,28 @@
           <t>multivitamin</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="C26" s="3" t="n">
         <v>1.27</v>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="D26" s="3" t="n">
         <v>1.04</v>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="E26" s="3" t="n">
         <v>1.56</v>
       </c>
-      <c r="F26" s="4" t="inlineStr"/>
-      <c r="G26" s="4" t="inlineStr"/>
-      <c r="H26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="6" t="inlineStr"/>
-      <c r="J26" s="3" t="n">
+      <c r="F26" s="3" t="inlineStr"/>
+      <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="5" t="inlineStr"/>
+      <c r="J26" s="2" t="n">
         <v>343481</v>
       </c>
-      <c r="K26" s="3" t="n">
+      <c r="K26" s="2" t="n">
         <v>2040</v>
       </c>
     </row>
@@ -1309,34 +1297,34 @@
           <t>alcohol</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B27" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C27" s="3" t="n">
         <v>1.28</v>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="D27" s="3" t="n">
         <v>0.73</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E27" s="3" t="n">
         <v>2.26</v>
       </c>
-      <c r="F27" s="4" t="n">
+      <c r="F27" s="3" t="n">
         <v>0.11</v>
       </c>
-      <c r="G27" s="4" t="n">
+      <c r="G27" s="3" t="n">
         <v>15.55</v>
       </c>
-      <c r="H27" s="5" t="n">
+      <c r="H27" s="4" t="n">
         <v>80</v>
       </c>
-      <c r="I27" s="6" t="n">
+      <c r="I27" s="5" t="n">
         <v>0.4695295847551806</v>
       </c>
-      <c r="J27" s="3" t="n">
+      <c r="J27" s="2" t="n">
         <v>166503</v>
       </c>
-      <c r="K27" s="3" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1344,28 +1332,28 @@
           <t>eggs</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C28" s="4" t="n">
+      <c r="C28" s="3" t="n">
         <v>1.36</v>
       </c>
-      <c r="D28" s="4" t="n">
+      <c r="D28" s="3" t="n">
         <v>0.87</v>
       </c>
-      <c r="E28" s="4" t="n">
+      <c r="E28" s="3" t="n">
         <v>2.1</v>
       </c>
-      <c r="F28" s="4" t="inlineStr"/>
-      <c r="G28" s="4" t="inlineStr"/>
-      <c r="H28" s="5" t="n">
+      <c r="F28" s="3" t="inlineStr"/>
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="4" t="n">
         <v>71.40000000000001</v>
       </c>
-      <c r="I28" s="6" t="inlineStr"/>
-      <c r="J28" s="3" t="n">
+      <c r="I28" s="5" t="inlineStr"/>
+      <c r="J28" s="2" t="n">
         <v>869756</v>
       </c>
-      <c r="K28" s="3" t="n">
+      <c r="K28" s="2" t="n">
         <v>5123</v>
       </c>
     </row>
@@ -1375,34 +1363,34 @@
           <t>dairy</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n">
+      <c r="B29" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="3" t="n">
         <v>1.41</v>
       </c>
-      <c r="D29" s="4" t="n">
+      <c r="D29" s="3" t="n">
         <v>1.14</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" s="3" t="n">
         <v>1.75</v>
       </c>
-      <c r="F29" s="4" t="n">
+      <c r="F29" s="3" t="n">
         <v>0.35</v>
       </c>
-      <c r="G29" s="4" t="n">
+      <c r="G29" s="3" t="n">
         <v>5.75</v>
       </c>
-      <c r="H29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="6" t="n">
-        <v>0.5307497625636001</v>
-      </c>
-      <c r="J29" s="3" t="n">
+      <c r="H29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>0.5307497625636</v>
+      </c>
+      <c r="J29" s="2" t="n">
         <v>101926</v>
       </c>
-      <c r="K29" s="3" t="n">
+      <c r="K29" s="2" t="n">
         <v>744</v>
       </c>
     </row>
@@ -1412,34 +1400,34 @@
           <t>processed_meat_intake</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="C30" s="3" t="n">
         <v>1.41</v>
       </c>
-      <c r="D30" s="4" t="n">
+      <c r="D30" s="3" t="n">
         <v>1.21</v>
       </c>
-      <c r="E30" s="4" t="n">
+      <c r="E30" s="3" t="n">
         <v>1.65</v>
       </c>
-      <c r="F30" s="4" t="n">
+      <c r="F30" s="3" t="n">
         <v>1.01</v>
       </c>
-      <c r="G30" s="4" t="n">
+      <c r="G30" s="3" t="n">
         <v>1.98</v>
       </c>
-      <c r="H30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="6" t="n">
+      <c r="H30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="5" t="n">
         <v>0.1345284439434558</v>
       </c>
-      <c r="J30" s="3" t="n">
+      <c r="J30" s="2" t="n">
         <v>204990</v>
       </c>
-      <c r="K30" s="3" t="n">
+      <c r="K30" s="2" t="n">
         <v>2302</v>
       </c>
     </row>
@@ -1449,34 +1437,34 @@
           <t>red_meat</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B31" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C31" s="4" t="n">
+      <c r="C31" s="3" t="n">
         <v>1.44</v>
       </c>
-      <c r="D31" s="4" t="n">
+      <c r="D31" s="3" t="n">
         <v>1.13</v>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="E31" s="3" t="n">
         <v>1.84</v>
       </c>
-      <c r="F31" s="4" t="n">
+      <c r="F31" s="3" t="n">
         <v>0.92</v>
       </c>
-      <c r="G31" s="4" t="n">
+      <c r="G31" s="3" t="n">
         <v>2.27</v>
       </c>
-      <c r="H31" s="5" t="n">
+      <c r="H31" s="4" t="n">
         <v>6.6</v>
       </c>
-      <c r="I31" s="6" t="n">
-        <v>0.2205851782199695</v>
-      </c>
-      <c r="J31" s="3" t="n">
+      <c r="I31" s="5" t="n">
+        <v>0.2205851782199696</v>
+      </c>
+      <c r="J31" s="2" t="n">
         <v>129031</v>
       </c>
-      <c r="K31" s="3" t="n">
+      <c r="K31" s="2" t="n">
         <v>1575</v>
       </c>
     </row>
@@ -1486,28 +1474,28 @@
           <t>genistein</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C32" s="4" t="n">
+      <c r="C32" s="3" t="n">
         <v>1.51</v>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="D32" s="3" t="n">
         <v>1.02</v>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="E32" s="3" t="n">
         <v>2.22</v>
       </c>
-      <c r="F32" s="4" t="inlineStr"/>
-      <c r="G32" s="4" t="inlineStr"/>
-      <c r="H32" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="6" t="inlineStr"/>
-      <c r="J32" s="3" t="n">
+      <c r="F32" s="3" t="inlineStr"/>
+      <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="5" t="inlineStr"/>
+      <c r="J32" s="2" t="n">
         <v>27004</v>
       </c>
-      <c r="K32" s="3" t="n">
+      <c r="K32" s="2" t="n">
         <v>287</v>
       </c>
     </row>
@@ -1517,34 +1505,34 @@
           <t>calcium</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C33" s="3" t="n">
         <v>1.53</v>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D33" s="3" t="n">
         <v>0.98</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E33" s="3" t="n">
         <v>2.38</v>
       </c>
-      <c r="F33" s="4" t="n">
+      <c r="F33" s="3" t="n">
         <v>0.36</v>
       </c>
-      <c r="G33" s="4" t="n">
+      <c r="G33" s="3" t="n">
         <v>6.44</v>
       </c>
-      <c r="H33" s="5" t="n">
+      <c r="H33" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="I33" s="6" t="n">
+      <c r="I33" s="5" t="n">
         <v>0.9970484632921824</v>
       </c>
-      <c r="J33" s="3" t="n">
+      <c r="J33" s="2" t="n">
         <v>98931</v>
       </c>
-      <c r="K33" s="3" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1552,28 +1540,28 @@
           <t>mineral_supplements</t>
         </is>
       </c>
-      <c r="B34" s="3" t="n">
+      <c r="B34" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C34" s="4" t="n">
+      <c r="C34" s="3" t="n">
         <v>1.8</v>
       </c>
-      <c r="D34" s="4" t="n">
+      <c r="D34" s="3" t="n">
         <v>1.19</v>
       </c>
-      <c r="E34" s="4" t="n">
+      <c r="E34" s="3" t="n">
         <v>2.73</v>
       </c>
-      <c r="F34" s="4" t="inlineStr"/>
-      <c r="G34" s="4" t="inlineStr"/>
-      <c r="H34" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" s="6" t="inlineStr"/>
-      <c r="J34" s="3" t="n">
+      <c r="F34" s="3" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="5" t="inlineStr"/>
+      <c r="J34" s="2" t="n">
         <v>47240</v>
       </c>
-      <c r="K34" s="3" t="n">
+      <c r="K34" s="2" t="n">
         <v>1143</v>
       </c>
     </row>
@@ -1583,34 +1571,34 @@
           <t>alpha_linolenic_acid</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B35" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="C35" s="3" t="n">
         <v>1.85</v>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="D35" s="3" t="n">
         <v>1.03</v>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="E35" s="3" t="n">
         <v>3.31</v>
       </c>
-      <c r="F35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="4" t="n">
+      <c r="F35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="3" t="n">
         <v>2021.94</v>
       </c>
-      <c r="H35" s="5" t="n">
+      <c r="H35" s="4" t="n">
         <v>86</v>
       </c>
-      <c r="I35" s="6" t="n">
+      <c r="I35" s="5" t="n">
         <v>0.01966497897827825</v>
       </c>
-      <c r="J35" s="3" t="n">
+      <c r="J35" s="2" t="n">
         <v>383989</v>
       </c>
-      <c r="K35" s="3" t="n">
+      <c r="K35" s="2" t="n">
         <v>3504</v>
       </c>
     </row>
@@ -1620,28 +1608,28 @@
           <t>carnitine</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n">
+      <c r="B36" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C36" s="4" t="n">
+      <c r="C36" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D36" s="4" t="n">
+      <c r="D36" s="3" t="n">
         <v>1.13</v>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="E36" s="3" t="n">
         <v>3.56</v>
       </c>
-      <c r="F36" s="4" t="inlineStr"/>
-      <c r="G36" s="4" t="inlineStr"/>
-      <c r="H36" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="6" t="inlineStr"/>
-      <c r="J36" s="3" t="n">
+      <c r="F36" s="3" t="inlineStr"/>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="5" t="inlineStr"/>
+      <c r="J36" s="2" t="n">
         <v>692</v>
       </c>
-      <c r="K36" s="3" t="n">
+      <c r="K36" s="2" t="n">
         <v>173</v>
       </c>
     </row>
@@ -1651,28 +1639,28 @@
           <t>choline</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B37" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C37" s="4" t="n">
+      <c r="C37" s="3" t="n">
         <v>2.19</v>
       </c>
-      <c r="D37" s="4" t="n">
+      <c r="D37" s="3" t="n">
         <v>1.23</v>
       </c>
-      <c r="E37" s="4" t="n">
+      <c r="E37" s="3" t="n">
         <v>3.9</v>
       </c>
-      <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="4" t="inlineStr"/>
-      <c r="H37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="6" t="inlineStr"/>
-      <c r="J37" s="3" t="n">
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr"/>
+      <c r="H37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="5" t="inlineStr"/>
+      <c r="J37" s="2" t="n">
         <v>692</v>
       </c>
-      <c r="K37" s="3" t="n">
+      <c r="K37" s="2" t="n">
         <v>173</v>
       </c>
     </row>
@@ -1682,28 +1670,28 @@
           <t>monounsaturated_fat_mufa</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B38" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C38" s="4" t="n">
+      <c r="C38" s="3" t="n">
         <v>2.39</v>
       </c>
-      <c r="D38" s="4" t="n">
+      <c r="D38" s="3" t="n">
         <v>1.37</v>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="E38" s="3" t="n">
         <v>4.15</v>
       </c>
-      <c r="F38" s="4" t="inlineStr"/>
-      <c r="G38" s="4" t="inlineStr"/>
-      <c r="H38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="6" t="inlineStr"/>
-      <c r="J38" s="3" t="n">
+      <c r="F38" s="3" t="inlineStr"/>
+      <c r="G38" s="3" t="inlineStr"/>
+      <c r="H38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="5" t="inlineStr"/>
+      <c r="J38" s="2" t="n">
         <v>144473</v>
       </c>
-      <c r="K38" s="3" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1711,28 +1699,28 @@
           <t>polyunsaturated_fat_pufa</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n">
+      <c r="B39" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C39" s="4" t="n">
+      <c r="C39" s="3" t="n">
         <v>2.7</v>
       </c>
-      <c r="D39" s="4" t="n">
+      <c r="D39" s="3" t="n">
         <v>1.1</v>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="E39" s="3" t="n">
         <v>6.8</v>
       </c>
-      <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="4" t="inlineStr"/>
-      <c r="H39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="6" t="inlineStr"/>
-      <c r="J39" s="3" t="n">
+      <c r="F39" s="3" t="inlineStr"/>
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="5" t="inlineStr"/>
+      <c r="J39" s="2" t="n">
         <v>721149</v>
       </c>
-      <c r="K39" s="3" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1740,28 +1728,28 @@
           <t>omega_3_fatty_acids</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B40" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C40" s="4" t="n">
+      <c r="C40" s="3" t="n">
         <v>3.43</v>
       </c>
-      <c r="D40" s="4" t="n">
+      <c r="D40" s="3" t="n">
         <v>1.67</v>
       </c>
-      <c r="E40" s="4" t="n">
+      <c r="E40" s="3" t="n">
         <v>7.04</v>
       </c>
-      <c r="F40" s="4" t="inlineStr"/>
-      <c r="G40" s="4" t="inlineStr"/>
-      <c r="H40" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" s="6" t="inlineStr"/>
-      <c r="J40" s="3" t="n">
+      <c r="F40" s="3" t="inlineStr"/>
+      <c r="G40" s="3" t="inlineStr"/>
+      <c r="H40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="5" t="inlineStr"/>
+      <c r="J40" s="2" t="n">
         <v>720112</v>
       </c>
-      <c r="K40" s="3" t="n">
+      <c r="K40" s="2" t="n">
         <v>4355</v>
       </c>
     </row>

</xml_diff>